<commit_message>
4Dash 1.1: exportar PNG/SVG/PDF, estilos de maquetación, zoom y licencia
- Barra de herramientas compacta de una fila que se adapta al zoom del
  navegador; paneles flotantes en ventanas estrechas; zoom −/+ y Ctrl+rueda.
- Exportar el dashboard tal y como se ve en el Presentador a PNG, SVG o PDF.
- Selector de color HTML libre en paletas y por serie de cada visual.
- Pestaña Estilo: estilos rápidos, rellenos sólidos y degradados, bordes,
  sombras, título, tipografía, grosor de línea, curvas, barras, anillo y
  fondo de página; nuevo visual Forma.
- Identidad visual propia (tokens, marca, favicon), textos sin referencias a
  productos de terceros y avisos de licencia de los iconos.
- Licencia 4Dash: uso comercial solo con atribución clara al autor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/datos_dummy.xlsx
+++ b/samples/datos_dummy.xlsx
@@ -76,7 +76,7 @@
     <t>Formación</t>
   </si>
   <si>
-    <t>Certificación Azure</t>
+    <t>Certificación en la nube</t>
   </si>
   <si>
     <t>Cyberdyne S.A.</t>
@@ -178,7 +178,7 @@
     <t>Raúl Gómez</t>
   </si>
   <si>
-    <t>Taller Excel avanzado</t>
+    <t>Taller de hojas de cálculo</t>
   </si>
   <si>
     <t>Globex S.A.</t>
@@ -187,7 +187,7 @@
     <t>Wonka S.L.</t>
   </si>
   <si>
-    <t>Curso Power BI</t>
+    <t>Curso de análisis de datos</t>
   </si>
   <si>
     <t>Jorge Sánchez</t>

</xml_diff>